<commit_message>
Make RM and FP analyst questionnaires self-contained
Respondent-facing text no longer names the feed files (study, Leadtime,
rawmaterials, database) or their sheets; the Questions sheet drops the
study-mapping column. Column order is unchanged for paste-back.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questionnaires/FP_Analyst_Questionnaire.xlsx
+++ b/questionnaires/FP_Analyst_Questionnaire.xlsx
@@ -636,7 +636,7 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>107 products in 64 method families and 385 family x test rows from QC_Capacity_Study.xlsx (Products, Test_Times).</t>
+          <t>107 products in 64 method families and 385 family x test rows.</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>7 families have no active ingredient in the formula database (F22, F37, F41, F42, F60, F62, F63) - name the actives in Test times Notes.</t>
+          <t>7 families have no active ingredient in the product formulas (F22, F37, F41, F42, F60, F62, F63) - name the actives in Test times Notes.</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>No recorded finished-product test times exist yet (Leadtime.xlsx covers raw materials only), so all times are new estimates.</t>
+          <t>No recorded finished-product test times exist yet (lab records cover raw materials only), so all times are new estimates.</t>
         </is>
       </c>
     </row>
@@ -715,13 +715,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D32"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
     <col width="70" customWidth="1" min="2" max="2"/>
     <col width="60" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -754,11 +753,6 @@
           <t>Answer</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>Feeds study sheet / column</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
@@ -768,7 +762,6 @@
       </c>
       <c r="B5" s="8" t="n"/>
       <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="9" t="inlineStr">
@@ -782,11 +775,6 @@
         </is>
       </c>
       <c r="C6" s="5" t="n"/>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Personnel A, B, D</t>
-        </is>
-      </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="9" t="inlineStr">
@@ -800,11 +788,6 @@
         </is>
       </c>
       <c r="C7" s="5" t="n"/>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>Personnel C; Test_Times X</t>
-        </is>
-      </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="9" t="inlineStr">
@@ -818,11 +801,6 @@
         </is>
       </c>
       <c r="C8" s="5" t="n"/>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Personnel E, F</t>
-        </is>
-      </c>
     </row>
     <row r="9" ht="45" customHeight="1">
       <c r="A9" s="9" t="inlineStr">
@@ -836,11 +814,6 @@
         </is>
       </c>
       <c r="C9" s="5" t="n"/>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>Personnel G, H</t>
-        </is>
-      </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="9" t="inlineStr">
@@ -854,11 +827,6 @@
         </is>
       </c>
       <c r="C10" s="5" t="n"/>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Personnel J; Evidence H</t>
-        </is>
-      </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
@@ -872,11 +840,6 @@
         </is>
       </c>
       <c r="C11" s="5" t="n"/>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>Report: key-person risk</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -886,7 +849,6 @@
       </c>
       <c r="B12" s="8" t="n"/>
       <c r="C12" s="8" t="n"/>
-      <c r="D12" s="8" t="n"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
@@ -900,11 +862,6 @@
         </is>
       </c>
       <c r="C13" s="5" t="n"/>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>Products F, I</t>
-        </is>
-      </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
@@ -918,11 +875,6 @@
         </is>
       </c>
       <c r="C14" s="5" t="n"/>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Products G, J</t>
-        </is>
-      </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
@@ -936,11 +888,6 @@
         </is>
       </c>
       <c r="C15" s="5" t="n"/>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>Extra tests</t>
-        </is>
-      </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
@@ -954,11 +901,6 @@
         </is>
       </c>
       <c r="C16" s="5" t="n"/>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Capacity C</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
@@ -968,7 +910,6 @@
       </c>
       <c r="B17" s="8" t="n"/>
       <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
@@ -982,11 +923,6 @@
         </is>
       </c>
       <c r="C18" s="5" t="n"/>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Test_Times J</t>
-        </is>
-      </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
@@ -1000,11 +936,6 @@
         </is>
       </c>
       <c r="C19" s="5" t="n"/>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>Test_Times G, R</t>
-        </is>
-      </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
@@ -1018,11 +949,6 @@
         </is>
       </c>
       <c r="C20" s="5" t="n"/>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>Test_Times U, J</t>
-        </is>
-      </c>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
@@ -1036,11 +962,6 @@
         </is>
       </c>
       <c r="C21" s="5" t="n"/>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>Test_Times I</t>
-        </is>
-      </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
@@ -1054,11 +975,6 @@
         </is>
       </c>
       <c r="C22" s="5" t="n"/>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Settings downtime</t>
-        </is>
-      </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
@@ -1072,11 +988,6 @@
         </is>
       </c>
       <c r="C23" s="5" t="n"/>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Settings hours/day</t>
-        </is>
-      </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
@@ -1090,11 +1001,6 @@
         </is>
       </c>
       <c r="C24" s="5" t="n"/>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Evidence; Notes</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
@@ -1104,7 +1010,6 @@
       </c>
       <c r="B25" s="8" t="n"/>
       <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
@@ -1118,11 +1023,6 @@
         </is>
       </c>
       <c r="C26" s="5" t="n"/>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>Evidence E, F, G</t>
-        </is>
-      </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
@@ -1136,11 +1036,6 @@
         </is>
       </c>
       <c r="C27" s="5" t="n"/>
-      <c r="D27" s="9" t="inlineStr">
-        <is>
-          <t>Evidence D, K</t>
-        </is>
-      </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
@@ -1154,11 +1049,6 @@
         </is>
       </c>
       <c r="C28" s="5" t="n"/>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>Capacity C</t>
-        </is>
-      </c>
     </row>
     <row r="29" ht="30" customHeight="1">
       <c r="A29" s="9" t="inlineStr">
@@ -1172,11 +1062,6 @@
         </is>
       </c>
       <c r="C29" s="5" t="n"/>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>Products; Settings growth</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
@@ -1186,7 +1071,6 @@
       </c>
       <c r="B30" s="8" t="n"/>
       <c r="C30" s="8" t="n"/>
-      <c r="D30" s="8" t="n"/>
     </row>
     <row r="31" ht="30" customHeight="1">
       <c r="A31" s="9" t="inlineStr">
@@ -1200,11 +1084,6 @@
         </is>
       </c>
       <c r="C31" s="5" t="n"/>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>Report_Outline</t>
-        </is>
-      </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="9" t="inlineStr">
@@ -1218,11 +1097,6 @@
         </is>
       </c>
       <c r="C32" s="5" t="n"/>
-      <c r="D32" s="9" t="inlineStr">
-        <is>
-          <t>Report_Outline</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1265,7 +1139,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Columns A-M = Products sheet of the study. Grey columns K-L are calculated in the study.</t>
+          <t>One row per product. Leave the narrow grey columns K-L empty.</t>
         </is>
       </c>
     </row>
@@ -1277,7 +1151,7 @@
       </c>
       <c r="B4" s="10" t="inlineStr">
         <is>
-          <t>Active(s) (from database)</t>
+          <t>Active(s) (from product formulas)</t>
         </is>
       </c>
       <c r="C4" s="10" t="inlineStr">
@@ -1337,7 +1211,7 @@
       </c>
       <c r="N4" s="10" t="inlineStr">
         <is>
-          <t>Stability time points / yr per batch on study</t>
+          <t>Stability time points / yr per batch on stability</t>
         </is>
       </c>
       <c r="O4" s="10" t="inlineStr">
@@ -3070,7 +2944,7 @@
       </c>
       <c r="B49" s="9" t="inlineStr">
         <is>
-          <t>Not in source file – define</t>
+          <t>Not on record – define</t>
         </is>
       </c>
       <c r="C49" s="9" t="n">
@@ -3655,7 +3529,7 @@
       </c>
       <c r="B64" s="9" t="inlineStr">
         <is>
-          <t>Not in source file – define</t>
+          <t>Not on record – define</t>
         </is>
       </c>
       <c r="C64" s="9" t="n">
@@ -4201,7 +4075,7 @@
       </c>
       <c r="B78" s="9" t="inlineStr">
         <is>
-          <t>Not in source file – define</t>
+          <t>Not on record – define</t>
         </is>
       </c>
       <c r="C78" s="9" t="n">
@@ -4357,7 +4231,7 @@
       </c>
       <c r="B82" s="9" t="inlineStr">
         <is>
-          <t>Not in source file – define</t>
+          <t>Not on record – define</t>
         </is>
       </c>
       <c r="C82" s="9" t="n">
@@ -4396,7 +4270,7 @@
       </c>
       <c r="B83" s="9" t="inlineStr">
         <is>
-          <t>Not in source file – define</t>
+          <t>Not on record – define</t>
         </is>
       </c>
       <c r="C83" s="9" t="n">
@@ -5293,7 +5167,7 @@
       </c>
       <c r="B106" s="9" t="inlineStr">
         <is>
-          <t>Not in source file – define</t>
+          <t>Not on record – define</t>
         </is>
       </c>
       <c r="C106" s="9" t="n">
@@ -5371,7 +5245,7 @@
       </c>
       <c r="B108" s="9" t="inlineStr">
         <is>
-          <t>Not in source file – define</t>
+          <t>Not on record – define</t>
         </is>
       </c>
       <c r="C108" s="9" t="n">
@@ -5410,7 +5284,7 @@
       </c>
       <c r="B109" s="9" t="inlineStr">
         <is>
-          <t>Not in source file – define</t>
+          <t>Not on record – define</t>
         </is>
       </c>
       <c r="C109" s="9" t="n">
@@ -5580,7 +5454,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>• Columns A-Z are in the same order as the Test_Times sheet of QC_Capacity_Study.xlsx: answers are pasted back 1:1.</t>
+          <t>• Do not insert, delete or reorder columns - the answers are collected by column position.</t>
         </is>
       </c>
     </row>
@@ -13663,7 +13537,7 @@
       <c r="Y136" s="5" t="n"/>
       <c r="Z136" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -13729,7 +13603,7 @@
       <c r="Y137" s="5" t="n"/>
       <c r="Z137" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -13795,7 +13669,7 @@
       <c r="Y138" s="5" t="n"/>
       <c r="Z138" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -13861,7 +13735,7 @@
       <c r="Y139" s="5" t="n"/>
       <c r="Z139" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -13927,7 +13801,7 @@
       <c r="Y140" s="5" t="n"/>
       <c r="Z140" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -13993,7 +13867,7 @@
       <c r="Y141" s="5" t="n"/>
       <c r="Z141" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -19275,7 +19149,7 @@
       <c r="Y226" s="5" t="n"/>
       <c r="Z226" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -19341,7 +19215,7 @@
       <c r="Y227" s="5" t="n"/>
       <c r="Z227" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -19407,7 +19281,7 @@
       <c r="Y228" s="5" t="n"/>
       <c r="Z228" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -19473,7 +19347,7 @@
       <c r="Y229" s="5" t="n"/>
       <c r="Z229" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -19539,7 +19413,7 @@
       <c r="Y230" s="5" t="n"/>
       <c r="Z230" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -19605,7 +19479,7 @@
       <c r="Y231" s="5" t="n"/>
       <c r="Z231" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -20791,7 +20665,7 @@
       <c r="Y250" s="5" t="n"/>
       <c r="Z250" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -20857,7 +20731,7 @@
       <c r="Y251" s="5" t="n"/>
       <c r="Z251" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -20923,7 +20797,7 @@
       <c r="Y252" s="5" t="n"/>
       <c r="Z252" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -20989,7 +20863,7 @@
       <c r="Y253" s="5" t="n"/>
       <c r="Z253" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -21055,7 +20929,7 @@
       <c r="Y254" s="5" t="n"/>
       <c r="Z254" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -21121,7 +20995,7 @@
       <c r="Y255" s="5" t="n"/>
       <c r="Z255" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -21187,7 +21061,7 @@
       <c r="Y256" s="5" t="n"/>
       <c r="Z256" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -21253,7 +21127,7 @@
       <c r="Y257" s="5" t="n"/>
       <c r="Z257" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -21319,7 +21193,7 @@
       <c r="Y258" s="5" t="n"/>
       <c r="Z258" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -21385,7 +21259,7 @@
       <c r="Y259" s="5" t="n"/>
       <c r="Z259" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -21451,7 +21325,7 @@
       <c r="Y260" s="5" t="n"/>
       <c r="Z260" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -21517,7 +21391,7 @@
       <c r="Y261" s="5" t="n"/>
       <c r="Z261" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -27951,7 +27825,7 @@
       <c r="Y364" s="5" t="n"/>
       <c r="Z364" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -28017,7 +27891,7 @@
       <c r="Y365" s="5" t="n"/>
       <c r="Z365" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -28083,7 +27957,7 @@
       <c r="Y366" s="5" t="n"/>
       <c r="Z366" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -28149,7 +28023,7 @@
       <c r="Y367" s="5" t="n"/>
       <c r="Z367" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -28215,7 +28089,7 @@
       <c r="Y368" s="5" t="n"/>
       <c r="Z368" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -28281,7 +28155,7 @@
       <c r="Y369" s="5" t="n"/>
       <c r="Z369" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -28719,7 +28593,7 @@
       <c r="Y376" s="5" t="n"/>
       <c r="Z376" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -28785,7 +28659,7 @@
       <c r="Y377" s="5" t="n"/>
       <c r="Z377" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -28851,7 +28725,7 @@
       <c r="Y378" s="5" t="n"/>
       <c r="Z378" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -28917,7 +28791,7 @@
       <c r="Y379" s="5" t="n"/>
       <c r="Z379" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -28983,7 +28857,7 @@
       <c r="Y380" s="5" t="n"/>
       <c r="Z380" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -29049,7 +28923,7 @@
       <c r="Y381" s="5" t="n"/>
       <c r="Z381" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -29115,7 +28989,7 @@
       <c r="Y382" s="5" t="n"/>
       <c r="Z382" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -29181,7 +29055,7 @@
       <c r="Y383" s="5" t="n"/>
       <c r="Z383" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -29247,7 +29121,7 @@
       <c r="Y384" s="5" t="n"/>
       <c r="Z384" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -29313,7 +29187,7 @@
       <c r="Y385" s="5" t="n"/>
       <c r="Z385" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -29379,7 +29253,7 @@
       <c r="Y386" s="5" t="n"/>
       <c r="Z386" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>
@@ -29445,7 +29319,7 @@
       <c r="Y387" s="5" t="n"/>
       <c r="Z387" s="5" t="inlineStr">
         <is>
-          <t>Actives not in source file – confirm tests</t>
+          <t>Actives not on record – confirm tests</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grey out questionnaire rows when Applicable = N or Outsourced = Y
Conditional formatting on Test times and Extra tests (RM and FP), and on the
RM Test catalog for outsourced tests; noted in the Guide colour rule.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/questionnaires/FP_Analyst_Questionnaire.xlsx
+++ b/questionnaires/FP_Analyst_Questionnaire.xlsx
@@ -146,6 +146,19 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="007F7F7F"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00BFBFBF"/>
+          <bgColor rgb="00BFBFBF"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -766,7 +779,7 @@
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>Yellow = you type. Grey = pre-filled or automatic; type over a grey value only if it is wrong.</t>
+          <t>Yellow = you type. Grey = pre-filled or automatic; type over a grey value only if it is wrong. Dark-grey row = Applicable = N or Outsourced = Y (outsourced rows still take the in-house Prep time).</t>
         </is>
       </c>
     </row>
@@ -33780,6 +33793,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AA386"/>
+  <conditionalFormatting sqref="A2:AA586">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>OR($F2="N",$AA2="Y")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="6">
     <dataValidation sqref="F2:F586" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
@@ -35835,6 +35853,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:AA41"/>
+  <conditionalFormatting sqref="A2:AA241">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="0">
+      <formula>OR($F2="N",$AA2="Y")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="6">
     <dataValidation sqref="F2:F241" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>

</xml_diff>